<commit_message>
Add Selenium E2E and Vulnerability reports generation
</commit_message>
<xml_diff>
--- a/test/E2E_TEST_Build.xlsx
+++ b/test/E2E_TEST_Build.xlsx
@@ -527,7 +527,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Functional Testing</t>
+          <t>Appium E2E Functional Testing</t>
         </is>
       </c>
     </row>
@@ -539,7 +539,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Flutter Web and Mobile</t>
+          <t>Flutter Mobile</t>
         </is>
       </c>
     </row>
@@ -1765,7 +1765,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1807,7 +1807,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -1849,7 +1849,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1886,12 +1886,12 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1970,12 +1970,12 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -2012,12 +2012,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2054,12 +2054,12 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2138,12 +2138,12 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -2306,12 +2306,12 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -2353,7 +2353,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -2390,12 +2390,12 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -2432,12 +2432,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2474,12 +2474,12 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -2521,7 +2521,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2558,12 +2558,12 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -2689,7 +2689,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2726,12 +2726,12 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -2773,7 +2773,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -2810,12 +2810,12 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -2852,12 +2852,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -2894,12 +2894,12 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -2941,7 +2941,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -2978,12 +2978,12 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -3025,7 +3025,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3146,12 +3146,12 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -3193,7 +3193,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -3230,12 +3230,12 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -3272,12 +3272,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -3314,12 +3314,12 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
@@ -3361,7 +3361,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -3398,12 +3398,12 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
@@ -3445,7 +3445,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -3529,7 +3529,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -3566,12 +3566,12 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
@@ -3613,7 +3613,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -3650,12 +3650,12 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
@@ -3692,12 +3692,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -3734,12 +3734,12 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
@@ -3781,7 +3781,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -3818,12 +3818,12 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
@@ -3865,7 +3865,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -3907,7 +3907,7 @@
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
@@ -3949,7 +3949,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -3986,12 +3986,12 @@
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -4070,12 +4070,12 @@
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
@@ -4112,12 +4112,12 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -4154,12 +4154,12 @@
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
@@ -4201,7 +4201,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -4238,12 +4238,12 @@
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
@@ -4285,7 +4285,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -4327,7 +4327,7 @@
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
@@ -4369,7 +4369,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -4406,12 +4406,12 @@
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
@@ -4453,7 +4453,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -4490,12 +4490,12 @@
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
@@ -4532,12 +4532,12 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -4574,12 +4574,12 @@
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
@@ -4621,7 +4621,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -4658,12 +4658,12 @@
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
@@ -4705,7 +4705,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -4747,7 +4747,7 @@
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr">
@@ -4789,7 +4789,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -4826,12 +4826,12 @@
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
@@ -4873,7 +4873,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -4910,12 +4910,12 @@
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
@@ -4952,12 +4952,12 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -4994,12 +4994,12 @@
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G79" s="3" t="inlineStr">
@@ -5041,7 +5041,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -5078,12 +5078,12 @@
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -5125,7 +5125,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -5167,7 +5167,7 @@
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
@@ -5209,7 +5209,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -5246,12 +5246,12 @@
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G85" s="3" t="inlineStr">
@@ -5293,7 +5293,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -5330,12 +5330,12 @@
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
@@ -5372,12 +5372,12 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -5414,12 +5414,12 @@
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G89" s="3" t="inlineStr">
@@ -5461,7 +5461,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -5498,12 +5498,12 @@
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G91" s="3" t="inlineStr">
@@ -5545,7 +5545,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -5587,7 +5587,7 @@
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G93" s="3" t="inlineStr">
@@ -5629,7 +5629,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -5666,12 +5666,12 @@
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G95" s="3" t="inlineStr">
@@ -5713,7 +5713,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -5750,12 +5750,12 @@
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G97" s="3" t="inlineStr">
@@ -5792,12 +5792,12 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -5834,12 +5834,12 @@
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G99" s="3" t="inlineStr">
@@ -5881,7 +5881,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -5918,12 +5918,12 @@
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G101" s="3" t="inlineStr">
@@ -5965,7 +5965,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -6007,7 +6007,7 @@
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G103" s="3" t="inlineStr">
@@ -6049,7 +6049,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -6086,12 +6086,12 @@
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G105" s="3" t="inlineStr">
@@ -6133,7 +6133,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -6170,12 +6170,12 @@
       </c>
       <c r="E107" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F107" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G107" s="3" t="inlineStr">
@@ -6212,12 +6212,12 @@
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -6254,12 +6254,12 @@
       </c>
       <c r="E109" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F109" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G109" s="3" t="inlineStr">
@@ -6301,7 +6301,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -6338,12 +6338,12 @@
       </c>
       <c r="E111" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F111" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G111" s="3" t="inlineStr">
@@ -6385,7 +6385,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -6427,7 +6427,7 @@
       </c>
       <c r="F113" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G113" s="3" t="inlineStr">
@@ -6469,7 +6469,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -6506,12 +6506,12 @@
       </c>
       <c r="E115" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F115" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G115" s="3" t="inlineStr">
@@ -6553,7 +6553,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -6590,12 +6590,12 @@
       </c>
       <c r="E117" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F117" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G117" s="3" t="inlineStr">
@@ -6632,12 +6632,12 @@
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -6674,12 +6674,12 @@
       </c>
       <c r="E119" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F119" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G119" s="3" t="inlineStr">
@@ -6721,7 +6721,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -6758,12 +6758,12 @@
       </c>
       <c r="E121" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F121" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G121" s="3" t="inlineStr">
@@ -6805,7 +6805,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -6847,7 +6847,7 @@
       </c>
       <c r="F123" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G123" s="3" t="inlineStr">
@@ -6889,7 +6889,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -6926,12 +6926,12 @@
       </c>
       <c r="E125" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F125" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G125" s="3" t="inlineStr">
@@ -6973,7 +6973,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -7010,12 +7010,12 @@
       </c>
       <c r="E127" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F127" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G127" s="3" t="inlineStr">
@@ -7052,12 +7052,12 @@
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -7094,12 +7094,12 @@
       </c>
       <c r="E129" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F129" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G129" s="3" t="inlineStr">
@@ -7141,7 +7141,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -7178,12 +7178,12 @@
       </c>
       <c r="E131" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F131" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G131" s="3" t="inlineStr">
@@ -7225,7 +7225,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -7267,7 +7267,7 @@
       </c>
       <c r="F133" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G133" s="3" t="inlineStr">
@@ -7309,7 +7309,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -7346,12 +7346,12 @@
       </c>
       <c r="E135" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F135" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G135" s="3" t="inlineStr">
@@ -7393,7 +7393,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -7430,12 +7430,12 @@
       </c>
       <c r="E137" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F137" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G137" s="3" t="inlineStr">
@@ -7472,12 +7472,12 @@
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -7514,12 +7514,12 @@
       </c>
       <c r="E139" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F139" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G139" s="3" t="inlineStr">
@@ -7561,7 +7561,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -7598,12 +7598,12 @@
       </c>
       <c r="E141" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F141" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G141" s="3" t="inlineStr">
@@ -7645,7 +7645,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -7687,7 +7687,7 @@
       </c>
       <c r="F143" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G143" s="3" t="inlineStr">
@@ -7729,7 +7729,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -7766,12 +7766,12 @@
       </c>
       <c r="E145" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F145" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G145" s="3" t="inlineStr">
@@ -7813,7 +7813,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -7850,12 +7850,12 @@
       </c>
       <c r="E147" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F147" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G147" s="3" t="inlineStr">
@@ -7892,12 +7892,12 @@
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -7934,12 +7934,12 @@
       </c>
       <c r="E149" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F149" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G149" s="3" t="inlineStr">
@@ -7981,7 +7981,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -8018,12 +8018,12 @@
       </c>
       <c r="E151" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F151" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G151" s="3" t="inlineStr">
@@ -8065,7 +8065,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -8107,7 +8107,7 @@
       </c>
       <c r="F153" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G153" s="3" t="inlineStr">
@@ -8149,7 +8149,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -8186,12 +8186,12 @@
       </c>
       <c r="E155" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F155" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G155" s="3" t="inlineStr">
@@ -8233,7 +8233,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -8270,12 +8270,12 @@
       </c>
       <c r="E157" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F157" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G157" s="3" t="inlineStr">
@@ -8312,12 +8312,12 @@
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -8354,12 +8354,12 @@
       </c>
       <c r="E159" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F159" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G159" s="3" t="inlineStr">
@@ -8401,7 +8401,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -8438,12 +8438,12 @@
       </c>
       <c r="E161" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F161" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G161" s="3" t="inlineStr">
@@ -8485,7 +8485,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -8527,7 +8527,7 @@
       </c>
       <c r="F163" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G163" s="3" t="inlineStr">
@@ -8569,7 +8569,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -8606,12 +8606,12 @@
       </c>
       <c r="E165" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G165" s="3" t="inlineStr">
@@ -8653,7 +8653,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -8690,12 +8690,12 @@
       </c>
       <c r="E167" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F167" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G167" s="3" t="inlineStr">
@@ -8732,12 +8732,12 @@
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -8774,12 +8774,12 @@
       </c>
       <c r="E169" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F169" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G169" s="3" t="inlineStr">
@@ -8821,7 +8821,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -8858,12 +8858,12 @@
       </c>
       <c r="E171" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F171" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G171" s="3" t="inlineStr">
@@ -8905,7 +8905,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -8947,7 +8947,7 @@
       </c>
       <c r="F173" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G173" s="3" t="inlineStr">
@@ -8989,7 +8989,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -9026,12 +9026,12 @@
       </c>
       <c r="E175" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F175" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G175" s="3" t="inlineStr">
@@ -9073,7 +9073,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -9110,12 +9110,12 @@
       </c>
       <c r="E177" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F177" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G177" s="3" t="inlineStr">
@@ -9152,12 +9152,12 @@
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -9194,12 +9194,12 @@
       </c>
       <c r="E179" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F179" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G179" s="3" t="inlineStr">
@@ -9241,7 +9241,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -9278,12 +9278,12 @@
       </c>
       <c r="E181" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F181" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G181" s="3" t="inlineStr">
@@ -9325,7 +9325,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -9367,7 +9367,7 @@
       </c>
       <c r="F183" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G183" s="3" t="inlineStr">
@@ -9409,7 +9409,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -9446,12 +9446,12 @@
       </c>
       <c r="E185" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F185" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G185" s="3" t="inlineStr">
@@ -9493,7 +9493,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -9530,12 +9530,12 @@
       </c>
       <c r="E187" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F187" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G187" s="3" t="inlineStr">
@@ -9572,12 +9572,12 @@
       </c>
       <c r="E188" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -9614,12 +9614,12 @@
       </c>
       <c r="E189" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F189" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G189" s="3" t="inlineStr">
@@ -9661,7 +9661,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -9698,12 +9698,12 @@
       </c>
       <c r="E191" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F191" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G191" s="3" t="inlineStr">
@@ -9745,7 +9745,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -9787,7 +9787,7 @@
       </c>
       <c r="F193" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G193" s="3" t="inlineStr">
@@ -9829,7 +9829,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -9866,12 +9866,12 @@
       </c>
       <c r="E195" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F195" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G195" s="3" t="inlineStr">
@@ -9913,7 +9913,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -9950,12 +9950,12 @@
       </c>
       <c r="E197" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F197" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G197" s="3" t="inlineStr">
@@ -9992,12 +9992,12 @@
       </c>
       <c r="E198" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -10034,12 +10034,12 @@
       </c>
       <c r="E199" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F199" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G199" s="3" t="inlineStr">
@@ -10081,7 +10081,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -10118,12 +10118,12 @@
       </c>
       <c r="E201" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F201" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G201" s="3" t="inlineStr">
@@ -10165,7 +10165,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -10207,7 +10207,7 @@
       </c>
       <c r="F203" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G203" s="3" t="inlineStr">
@@ -10249,7 +10249,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -10286,12 +10286,12 @@
       </c>
       <c r="E205" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F205" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G205" s="3" t="inlineStr">
@@ -10333,7 +10333,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -10370,12 +10370,12 @@
       </c>
       <c r="E207" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F207" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G207" s="3" t="inlineStr">
@@ -10412,12 +10412,12 @@
       </c>
       <c r="E208" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -10454,12 +10454,12 @@
       </c>
       <c r="E209" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F209" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G209" s="3" t="inlineStr">
@@ -10501,7 +10501,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -10538,12 +10538,12 @@
       </c>
       <c r="E211" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F211" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G211" s="3" t="inlineStr">
@@ -10585,7 +10585,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -10627,7 +10627,7 @@
       </c>
       <c r="F213" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G213" s="3" t="inlineStr">
@@ -10669,7 +10669,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -10706,12 +10706,12 @@
       </c>
       <c r="E215" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F215" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G215" s="3" t="inlineStr">
@@ -10753,7 +10753,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -10790,12 +10790,12 @@
       </c>
       <c r="E217" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F217" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G217" s="3" t="inlineStr">
@@ -10832,12 +10832,12 @@
       </c>
       <c r="E218" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -10874,12 +10874,12 @@
       </c>
       <c r="E219" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F219" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G219" s="3" t="inlineStr">
@@ -10921,7 +10921,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -10958,12 +10958,12 @@
       </c>
       <c r="E221" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F221" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G221" s="3" t="inlineStr">
@@ -11005,7 +11005,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
@@ -11047,7 +11047,7 @@
       </c>
       <c r="F223" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G223" s="3" t="inlineStr">
@@ -11089,7 +11089,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -11126,12 +11126,12 @@
       </c>
       <c r="E225" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F225" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G225" s="3" t="inlineStr">
@@ -11173,7 +11173,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -11210,12 +11210,12 @@
       </c>
       <c r="E227" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F227" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G227" s="3" t="inlineStr">
@@ -11252,12 +11252,12 @@
       </c>
       <c r="E228" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
@@ -11294,12 +11294,12 @@
       </c>
       <c r="E229" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F229" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G229" s="3" t="inlineStr">
@@ -11341,7 +11341,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -11378,12 +11378,12 @@
       </c>
       <c r="E231" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F231" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G231" s="3" t="inlineStr">
@@ -11425,7 +11425,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -11467,7 +11467,7 @@
       </c>
       <c r="F233" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G233" s="3" t="inlineStr">
@@ -11509,7 +11509,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -11546,12 +11546,12 @@
       </c>
       <c r="E235" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F235" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G235" s="3" t="inlineStr">
@@ -11593,7 +11593,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -11630,12 +11630,12 @@
       </c>
       <c r="E237" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F237" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G237" s="3" t="inlineStr">
@@ -11672,12 +11672,12 @@
       </c>
       <c r="E238" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -11714,12 +11714,12 @@
       </c>
       <c r="E239" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F239" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G239" s="3" t="inlineStr">
@@ -11761,7 +11761,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -11798,12 +11798,12 @@
       </c>
       <c r="E241" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F241" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G241" s="3" t="inlineStr">
@@ -11845,7 +11845,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -11887,7 +11887,7 @@
       </c>
       <c r="F243" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G243" s="3" t="inlineStr">
@@ -11929,7 +11929,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
@@ -11966,12 +11966,12 @@
       </c>
       <c r="E245" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F245" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G245" s="3" t="inlineStr">
@@ -12013,7 +12013,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -12050,12 +12050,12 @@
       </c>
       <c r="E247" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F247" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G247" s="3" t="inlineStr">
@@ -12092,12 +12092,12 @@
       </c>
       <c r="E248" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -12134,12 +12134,12 @@
       </c>
       <c r="E249" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F249" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G249" s="3" t="inlineStr">
@@ -12181,7 +12181,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -12218,12 +12218,12 @@
       </c>
       <c r="E251" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F251" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G251" s="3" t="inlineStr">
@@ -12265,7 +12265,7 @@
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
@@ -12307,7 +12307,7 @@
       </c>
       <c r="F253" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G253" s="3" t="inlineStr">
@@ -12349,7 +12349,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr">
@@ -12386,12 +12386,12 @@
       </c>
       <c r="E255" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F255" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G255" s="3" t="inlineStr">
@@ -12433,7 +12433,7 @@
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G256" s="2" t="inlineStr">
@@ -12470,12 +12470,12 @@
       </c>
       <c r="E257" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F257" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G257" s="3" t="inlineStr">
@@ -12512,12 +12512,12 @@
       </c>
       <c r="E258" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
@@ -12554,12 +12554,12 @@
       </c>
       <c r="E259" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F259" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G259" s="3" t="inlineStr">
@@ -12601,7 +12601,7 @@
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
@@ -12638,12 +12638,12 @@
       </c>
       <c r="E261" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F261" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G261" s="3" t="inlineStr">
@@ -12685,7 +12685,7 @@
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr">
@@ -12727,7 +12727,7 @@
       </c>
       <c r="F263" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G263" s="3" t="inlineStr">
@@ -12769,7 +12769,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
@@ -12806,12 +12806,12 @@
       </c>
       <c r="E265" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F265" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G265" s="3" t="inlineStr">
@@ -12853,7 +12853,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
@@ -12890,12 +12890,12 @@
       </c>
       <c r="E267" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F267" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G267" s="3" t="inlineStr">
@@ -12932,12 +12932,12 @@
       </c>
       <c r="E268" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G268" s="2" t="inlineStr">
@@ -12974,12 +12974,12 @@
       </c>
       <c r="E269" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F269" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G269" s="3" t="inlineStr">
@@ -13021,7 +13021,7 @@
       </c>
       <c r="F270" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G270" s="2" t="inlineStr">
@@ -13058,12 +13058,12 @@
       </c>
       <c r="E271" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F271" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G271" s="3" t="inlineStr">
@@ -13105,7 +13105,7 @@
       </c>
       <c r="F272" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G272" s="2" t="inlineStr">
@@ -13147,7 +13147,7 @@
       </c>
       <c r="F273" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G273" s="3" t="inlineStr">
@@ -13189,7 +13189,7 @@
       </c>
       <c r="F274" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G274" s="2" t="inlineStr">
@@ -13226,12 +13226,12 @@
       </c>
       <c r="E275" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F275" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G275" s="3" t="inlineStr">
@@ -13273,7 +13273,7 @@
       </c>
       <c r="F276" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G276" s="2" t="inlineStr">
@@ -13310,12 +13310,12 @@
       </c>
       <c r="E277" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F277" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G277" s="3" t="inlineStr">
@@ -13352,12 +13352,12 @@
       </c>
       <c r="E278" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F278" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G278" s="2" t="inlineStr">
@@ -13394,12 +13394,12 @@
       </c>
       <c r="E279" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F279" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G279" s="3" t="inlineStr">
@@ -13441,7 +13441,7 @@
       </c>
       <c r="F280" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G280" s="2" t="inlineStr">
@@ -13478,12 +13478,12 @@
       </c>
       <c r="E281" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F281" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G281" s="3" t="inlineStr">
@@ -13525,7 +13525,7 @@
       </c>
       <c r="F282" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G282" s="2" t="inlineStr">
@@ -13567,7 +13567,7 @@
       </c>
       <c r="F283" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G283" s="3" t="inlineStr">
@@ -13609,7 +13609,7 @@
       </c>
       <c r="F284" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G284" s="2" t="inlineStr">
@@ -13646,12 +13646,12 @@
       </c>
       <c r="E285" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F285" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G285" s="3" t="inlineStr">
@@ -13693,7 +13693,7 @@
       </c>
       <c r="F286" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G286" s="2" t="inlineStr">
@@ -13730,12 +13730,12 @@
       </c>
       <c r="E287" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F287" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G287" s="3" t="inlineStr">
@@ -13772,12 +13772,12 @@
       </c>
       <c r="E288" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F288" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G288" s="2" t="inlineStr">
@@ -13814,12 +13814,12 @@
       </c>
       <c r="E289" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F289" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G289" s="3" t="inlineStr">
@@ -13861,7 +13861,7 @@
       </c>
       <c r="F290" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G290" s="2" t="inlineStr">
@@ -13898,12 +13898,12 @@
       </c>
       <c r="E291" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F291" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G291" s="3" t="inlineStr">
@@ -13945,7 +13945,7 @@
       </c>
       <c r="F292" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G292" s="2" t="inlineStr">
@@ -13987,7 +13987,7 @@
       </c>
       <c r="F293" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G293" s="3" t="inlineStr">
@@ -14029,7 +14029,7 @@
       </c>
       <c r="F294" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G294" s="2" t="inlineStr">
@@ -14066,12 +14066,12 @@
       </c>
       <c r="E295" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F295" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G295" s="3" t="inlineStr">
@@ -14113,7 +14113,7 @@
       </c>
       <c r="F296" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G296" s="2" t="inlineStr">
@@ -14150,12 +14150,12 @@
       </c>
       <c r="E297" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F297" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G297" s="3" t="inlineStr">
@@ -14192,12 +14192,12 @@
       </c>
       <c r="E298" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F298" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G298" s="2" t="inlineStr">
@@ -14234,12 +14234,12 @@
       </c>
       <c r="E299" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F299" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G299" s="3" t="inlineStr">
@@ -14281,7 +14281,7 @@
       </c>
       <c r="F300" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G300" s="2" t="inlineStr">
@@ -14318,12 +14318,12 @@
       </c>
       <c r="E301" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F301" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G301" s="3" t="inlineStr">
@@ -14365,7 +14365,7 @@
       </c>
       <c r="F302" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G302" s="2" t="inlineStr">
@@ -14407,7 +14407,7 @@
       </c>
       <c r="F303" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G303" s="3" t="inlineStr">
@@ -14449,7 +14449,7 @@
       </c>
       <c r="F304" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G304" s="2" t="inlineStr">
@@ -14486,12 +14486,12 @@
       </c>
       <c r="E305" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F305" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G305" s="3" t="inlineStr">
@@ -14533,7 +14533,7 @@
       </c>
       <c r="F306" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G306" s="2" t="inlineStr">
@@ -14570,12 +14570,12 @@
       </c>
       <c r="E307" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F307" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G307" s="3" t="inlineStr">
@@ -14612,12 +14612,12 @@
       </c>
       <c r="E308" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F308" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G308" s="2" t="inlineStr">
@@ -14654,12 +14654,12 @@
       </c>
       <c r="E309" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F309" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G309" s="3" t="inlineStr">
@@ -14701,7 +14701,7 @@
       </c>
       <c r="F310" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G310" s="2" t="inlineStr">
@@ -14738,12 +14738,12 @@
       </c>
       <c r="E311" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F311" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G311" s="3" t="inlineStr">
@@ -14785,7 +14785,7 @@
       </c>
       <c r="F312" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G312" s="2" t="inlineStr">
@@ -14827,7 +14827,7 @@
       </c>
       <c r="F313" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G313" s="3" t="inlineStr">
@@ -14869,7 +14869,7 @@
       </c>
       <c r="F314" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G314" s="2" t="inlineStr">
@@ -14906,12 +14906,12 @@
       </c>
       <c r="E315" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F315" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G315" s="3" t="inlineStr">
@@ -14953,7 +14953,7 @@
       </c>
       <c r="F316" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G316" s="2" t="inlineStr">
@@ -14990,12 +14990,12 @@
       </c>
       <c r="E317" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F317" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G317" s="3" t="inlineStr">
@@ -15032,12 +15032,12 @@
       </c>
       <c r="E318" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F318" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G318" s="2" t="inlineStr">
@@ -15074,12 +15074,12 @@
       </c>
       <c r="E319" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F319" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G319" s="3" t="inlineStr">
@@ -15121,7 +15121,7 @@
       </c>
       <c r="F320" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G320" s="2" t="inlineStr">
@@ -15158,12 +15158,12 @@
       </c>
       <c r="E321" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F321" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G321" s="3" t="inlineStr">
@@ -15205,7 +15205,7 @@
       </c>
       <c r="F322" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G322" s="2" t="inlineStr">
@@ -15247,7 +15247,7 @@
       </c>
       <c r="F323" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G323" s="3" t="inlineStr">
@@ -15289,7 +15289,7 @@
       </c>
       <c r="F324" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G324" s="2" t="inlineStr">
@@ -15326,12 +15326,12 @@
       </c>
       <c r="E325" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F325" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G325" s="3" t="inlineStr">
@@ -15373,7 +15373,7 @@
       </c>
       <c r="F326" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G326" s="2" t="inlineStr">
@@ -15410,12 +15410,12 @@
       </c>
       <c r="E327" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F327" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G327" s="3" t="inlineStr">
@@ -15452,12 +15452,12 @@
       </c>
       <c r="E328" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F328" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G328" s="2" t="inlineStr">
@@ -15494,12 +15494,12 @@
       </c>
       <c r="E329" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F329" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G329" s="3" t="inlineStr">
@@ -15541,7 +15541,7 @@
       </c>
       <c r="F330" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G330" s="2" t="inlineStr">
@@ -15578,12 +15578,12 @@
       </c>
       <c r="E331" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F331" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G331" s="3" t="inlineStr">
@@ -15625,7 +15625,7 @@
       </c>
       <c r="F332" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G332" s="2" t="inlineStr">
@@ -15667,7 +15667,7 @@
       </c>
       <c r="F333" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G333" s="3" t="inlineStr">
@@ -15709,7 +15709,7 @@
       </c>
       <c r="F334" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G334" s="2" t="inlineStr">
@@ -15746,12 +15746,12 @@
       </c>
       <c r="E335" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F335" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G335" s="3" t="inlineStr">
@@ -15793,7 +15793,7 @@
       </c>
       <c r="F336" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G336" s="2" t="inlineStr">
@@ -15830,12 +15830,12 @@
       </c>
       <c r="E337" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F337" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G337" s="3" t="inlineStr">
@@ -15872,12 +15872,12 @@
       </c>
       <c r="E338" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F338" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G338" s="2" t="inlineStr">
@@ -15914,12 +15914,12 @@
       </c>
       <c r="E339" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F339" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G339" s="3" t="inlineStr">
@@ -15961,7 +15961,7 @@
       </c>
       <c r="F340" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G340" s="2" t="inlineStr">
@@ -15998,12 +15998,12 @@
       </c>
       <c r="E341" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F341" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G341" s="3" t="inlineStr">
@@ -16045,7 +16045,7 @@
       </c>
       <c r="F342" s="2" t="inlineStr">
         <is>
-          <t>The screen should load successfully without any errors or infinite loading indicators.</t>
+          <t>The screen should load successfully without any errors.</t>
         </is>
       </c>
       <c r="G342" s="2" t="inlineStr">
@@ -16087,7 +16087,7 @@
       </c>
       <c r="F343" s="3" t="inlineStr">
         <is>
-          <t>All UI elements should be clearly visible and correctly aligned.</t>
+          <t>All UI elements should be clearly visible.</t>
         </is>
       </c>
       <c r="G343" s="3" t="inlineStr">
@@ -16129,7 +16129,7 @@
       </c>
       <c r="F344" s="2" t="inlineStr">
         <is>
-          <t>Application should navigate to the correct subsequent screen or previous screen.</t>
+          <t>Application should navigate to the correct screen.</t>
         </is>
       </c>
       <c r="G344" s="2" t="inlineStr">
@@ -16166,12 +16166,12 @@
       </c>
       <c r="E345" s="3" t="inlineStr">
         <is>
-          <t>If applicable, enter valid and invalid data into input fields and submit.</t>
+          <t>Enter valid and invalid data into input fields.</t>
         </is>
       </c>
       <c r="F345" s="3" t="inlineStr">
         <is>
-          <t>System should accept valid data and show appropriate validation messages for invalid data.</t>
+          <t>System should accept valid data and show appropriate validation messages.</t>
         </is>
       </c>
       <c r="G345" s="3" t="inlineStr">
@@ -16213,7 +16213,7 @@
       </c>
       <c r="F346" s="2" t="inlineStr">
         <is>
-          <t>Buttons should trigger the expected action or open the relevant dialogs/modals.</t>
+          <t>Buttons should trigger the expected action.</t>
         </is>
       </c>
       <c r="G346" s="2" t="inlineStr">
@@ -16250,12 +16250,12 @@
       </c>
       <c r="E347" s="3" t="inlineStr">
         <is>
-          <t>Verify the data populated on the screen matches the backend or expected mock data.</t>
+          <t>Verify the data populated on the screen matches expected mock data.</t>
         </is>
       </c>
       <c r="F347" s="3" t="inlineStr">
         <is>
-          <t>Data displayed should be accurate and match the source without truncation.</t>
+          <t>Data displayed should be accurate.</t>
         </is>
       </c>
       <c r="G347" s="3" t="inlineStr">
@@ -16292,12 +16292,12 @@
       </c>
       <c r="E348" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error or API failure while performing an action.</t>
+          <t>Simulate a network error while performing an action.</t>
         </is>
       </c>
       <c r="F348" s="2" t="inlineStr">
         <is>
-          <t>System should gracefully handle the error and display a user-friendly error message.</t>
+          <t>System should display a user-friendly error message.</t>
         </is>
       </c>
       <c r="G348" s="2" t="inlineStr">
@@ -16334,12 +16334,12 @@
       </c>
       <c r="E349" s="3" t="inlineStr">
         <is>
-          <t>Resize the window or test on different device screen sizes.</t>
+          <t>Test on different device screen sizes.</t>
         </is>
       </c>
       <c r="F349" s="3" t="inlineStr">
         <is>
-          <t>Screen layout should adapt correctly without overlapping UI elements.</t>
+          <t>Screen layout should adapt correctly.</t>
         </is>
       </c>
       <c r="G349" s="3" t="inlineStr">
@@ -16381,7 +16381,7 @@
       </c>
       <c r="F350" s="2" t="inlineStr">
         <is>
-          <t>API requests should be sent correctly and data should be updated in the database.</t>
+          <t>API requests should be sent correctly.</t>
         </is>
       </c>
       <c r="G350" s="2" t="inlineStr">
@@ -16418,12 +16418,12 @@
       </c>
       <c r="E351" s="3" t="inlineStr">
         <is>
-          <t>Complete the primary workflow intended for this specific screen.</t>
+          <t>Complete the primary workflow.</t>
         </is>
       </c>
       <c r="F351" s="3" t="inlineStr">
         <is>
-          <t>The workflow should complete successfully, ending in the desired state.</t>
+          <t>The workflow should complete successfully.</t>
         </is>
       </c>
       <c r="G351" s="3" t="inlineStr">

</xml_diff>